<commit_message>
Clarified that by default only a selected few bout and percentile variables are generated.
</commit_message>
<xml_diff>
--- a/docs/Extra/ActiPASS_Variable-definitions_NewFormat_ActiPASS_Version_1.50.xlsx
+++ b/docs/Extra/ActiPASS_Variable-definitions_NewFormat_ActiPASS_Version_1.50.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28526"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29822"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\pashe866\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{00D09A24-2465-463B-95B4-9AA79042197F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8740E721-E5F2-429F-98E9-B326CF20E085}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -163,14 +163,7 @@
     <t>Cadence related variables. Cadence is only detected for walking, running and stair-walking</t>
   </si>
   <si>
-    <t>Important Note: These variables are calculated using the direct output of activity detection algorithm with an epoch of 1s. Any sporadic break, misclassification or ambiguity can affect these variables. These variables, except for the combined activity/posture "SitLie", should only be used with consultation of ActiPASS developers</t>
-  </si>
-  <si>
     <t>replace "SitLie" with the relevant activity/posture/intensity-class to derive corresponding variable name (also see warning above)</t>
-  </si>
-  <si>
-    <t>Important Note: If ProPASS default settings are applied, then these variables are calculated allowing a fixed bout-break of 20s with 0% bout thresholds. 
-However, if bout-calculations options are changed under advanced settings, different bout-break lengths and different bout-thresholds can be selected. Before generating these variables make sure desired settings are applied under ActiPASS advanced options</t>
   </si>
   <si>
     <t>Time spent on SitLie bouts  equal or larger than 1min</t>
@@ -493,115 +486,6 @@
   </si>
   <si>
     <t>QC_Status</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="5" tint="-0.499984740745262"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t>Bouts related variables of  activity/posture/intensity-classes.   The combined posture "SitLie" is chosen as an example. These Variables are also derived for following activity/postures as well as intensity classes.</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FFC00000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t>Lie, Sit, SitLie, Stand, Move, StandMove,  Walk, Run, Stair, Cycle, Upright, Other,INT1, INT2, INT2_Amb, INT3, INT4, INT34</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="5" tint="-0.499984740745262"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t>Time percentiles of continuous segments of activity/posture/intensity-classes  and breaks of activity/posture/intensity-classes.</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="5" tint="-0.499984740745262"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve"> </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">  </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="5" tint="-0.499984740745262"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">The posture </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="5" tint="-0.499984740745262"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t>"SitLie"</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="5" tint="-0.499984740745262"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve"> is chosen as an example. These Variables are also derived for following activity/postures as well as intensity classes.</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FFC00000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">Lie, Sit, SitLie, Stand, Move, StandMove,  Walk, Run, Stair, Cycle, Upright, Other, INT1, INT2, INT2_Amb, INT3, INT4, INT34
-</t>
-    </r>
   </si>
   <si>
     <r>
@@ -1373,12 +1257,329 @@
   <si>
     <t>Automatic individual calibration angles (in degrees) for this day. Given as absolute inclination and forward backward inclination of thigh at the reference-position</t>
   </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="5" tint="-0.499984740745262"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">Bouts related variables of  activity/posture/intensity-classes.   The combined posture "SitLie" is chosen as an example. These Variables could also derived for following activity/postures as well as intensity classes  (variables in </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="9" tint="-0.249977111117893"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>green</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="5" tint="-0.499984740745262"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> are generated by default). </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FFC00000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">Lie, Sit, </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="9" tint="-0.249977111117893"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>SitLie</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FFC00000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">, Stand, Move, StandMove,  Walk, Run, Stair, Cycle, </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="9" tint="-0.249977111117893"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>Upright</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FFC00000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">, Other,INT1, INT2, INT2_Amb, INT3, INT4, </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="9" tint="-0.249977111117893"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>INT34</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="5" tint="-0.499984740745262"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>Time percentiles of continuous segments of activity/posture/intensity-classes  and breaks of activity/posture/intensity-classes.</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="5" tint="-0.499984740745262"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">  </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="5" tint="-0.499984740745262"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">The posture </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="5" tint="-0.499984740745262"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>"SitLie"</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="5" tint="-0.499984740745262"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> is chosen as an example. These Variables could also be derived for following activity/postures as well as intensity classes (variables in green are generated by default). </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FFC00000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">Lie, Sit, </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="9" tint="-0.249977111117893"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>SitLie</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FFC00000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">, Stand, Move, StandMove,  Walk, Run, Stair, Cycle, </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="9" tint="-0.249977111117893"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>Upright</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FFC00000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">, Other, INT1, INT2, INT2_Amb, INT3, INT4, </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="9" tint="-0.249977111117893"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>INT34</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FFC00000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Important Note: These variables are calculated using the direct output of activity detection algorithm with an epoch of 1s. Any sporadic break, misclassification or ambiguity can affect these variables. 
+Additional percentile variables could be generated by enabling them in a configuration file. 
+See: 
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF0070C0"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>1. https://github.com/Ergo-Tools/ActiPASS/wiki/Adjusting-algorithm-parameters,-and-options-which-are-not-exposed-via-GUI</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Important Note: If ProPASS default settings are applied, then these variables are calculated allowing a fixed bout-break of 20s with 0% bout thresholds. 
+However, if bout-calculations options are changed under advanced settings, different bout-break lengths and different bout-thresholds can be selected. Before generating these variables make sure desired settings are applied under ActiPASS advanced options.
+Additional bout variables could be generated by enabling them in a configuration file. 
+See: 
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF0070C0"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>1. https://github.com/Ergo-Tools/ActiPASS/wiki/Adjusting-algorithm-parameters,-and-options-which-are-not-exposed-via-GUI</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FFC00000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF0070C0"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>2.</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FFC00000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF0070C0"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>https://github.com/Ergo-Tools/ActiPASS/wiki/How-bout-variables-are-derived-by-ActiPASS</t>
+    </r>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="26" x14ac:knownFonts="1">
+  <fonts count="28" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <name val="Calibri"/>
@@ -1550,6 +1751,20 @@
       <sz val="10"/>
       <name val="Times New Roman"/>
       <family val="1"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="9" tint="-0.249977111117893"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FF0070C0"/>
+      <name val="Calibri"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="6">
@@ -2103,7 +2318,7 @@
   <sheetData>
     <row r="1" spans="1:3" s="26" customFormat="1" ht="20.25" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A1" s="26" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="B1" s="27"/>
       <c r="C1" s="27"/>
@@ -2114,7 +2329,7 @@
     </row>
     <row r="3" spans="1:3" s="26" customFormat="1" ht="21" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A3" s="36" t="s">
-        <v>218</v>
+        <v>214</v>
       </c>
       <c r="B3" s="27"/>
       <c r="C3" s="27"/>
@@ -2141,13 +2356,13 @@
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="B7" s="10" t="s">
-        <v>116</v>
+        <v>112</v>
       </c>
       <c r="C7" s="10" t="s">
-        <v>117</v>
+        <v>113</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
@@ -2158,7 +2373,7 @@
         <v>9</v>
       </c>
       <c r="C8" s="10" t="s">
-        <v>217</v>
+        <v>213</v>
       </c>
     </row>
     <row r="9" spans="1:3" ht="30" x14ac:dyDescent="0.25">
@@ -2184,10 +2399,10 @@
         <v>5</v>
       </c>
       <c r="B11" s="30" t="s">
-        <v>118</v>
+        <v>114</v>
       </c>
       <c r="C11" s="31" t="s">
-        <v>119</v>
+        <v>115</v>
       </c>
     </row>
     <row r="12" spans="1:3" s="11" customFormat="1" ht="30" x14ac:dyDescent="0.25">
@@ -2195,18 +2410,18 @@
         <v>6</v>
       </c>
       <c r="B12" s="30" t="s">
-        <v>120</v>
+        <v>116</v>
       </c>
       <c r="C12" s="31" t="s">
-        <v>119</v>
+        <v>115</v>
       </c>
     </row>
     <row r="13" spans="1:3" s="17" customFormat="1" ht="71.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B13" s="28" t="s">
-        <v>215</v>
+        <v>211</v>
       </c>
       <c r="C13" s="32" t="s">
-        <v>242</v>
+        <v>238</v>
       </c>
     </row>
     <row r="14" spans="1:3" s="33" customFormat="1" ht="36" customHeight="1" x14ac:dyDescent="0.25">
@@ -2215,7 +2430,7 @@
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>121</v>
+        <v>117</v>
       </c>
       <c r="B15" s="4" t="s">
         <v>11</v>
@@ -2224,7 +2439,7 @@
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>122</v>
+        <v>118</v>
       </c>
       <c r="B16" s="4" t="s">
         <v>12</v>
@@ -2233,7 +2448,7 @@
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>123</v>
+        <v>119</v>
       </c>
       <c r="B17" s="4" t="s">
         <v>13</v>
@@ -2242,18 +2457,18 @@
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>124</v>
+        <v>120</v>
       </c>
       <c r="B18" s="10" t="s">
-        <v>114</v>
+        <v>110</v>
       </c>
       <c r="C18" s="10" t="s">
-        <v>115</v>
+        <v>111</v>
       </c>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>125</v>
+        <v>121</v>
       </c>
       <c r="B19" s="4" t="s">
         <v>14</v>
@@ -2262,7 +2477,7 @@
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>126</v>
+        <v>122</v>
       </c>
       <c r="B20" s="4" t="s">
         <v>15</v>
@@ -2271,99 +2486,99 @@
     </row>
     <row r="21" spans="1:3" ht="30" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>127</v>
+        <v>123</v>
       </c>
       <c r="B21" s="10" t="s">
-        <v>221</v>
+        <v>217</v>
       </c>
       <c r="C21" s="10" t="s">
-        <v>222</v>
+        <v>218</v>
       </c>
     </row>
     <row r="22" spans="1:3" ht="30" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>243</v>
+        <v>239</v>
       </c>
       <c r="B22" s="10" t="s">
-        <v>244</v>
+        <v>240</v>
       </c>
       <c r="C22" s="10"/>
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>128</v>
+        <v>124</v>
       </c>
       <c r="B23" s="10" t="s">
-        <v>219</v>
+        <v>215</v>
       </c>
       <c r="C23" s="10" t="s">
-        <v>220</v>
+        <v>216</v>
       </c>
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>129</v>
+        <v>125</v>
       </c>
       <c r="B24" s="10" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="C24" s="10" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
     </row>
     <row r="25" spans="1:3" ht="30" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>130</v>
+        <v>126</v>
       </c>
       <c r="B25" s="10" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="C25" s="10" t="s">
-        <v>230</v>
+        <v>226</v>
       </c>
     </row>
     <row r="26" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>131</v>
+        <v>127</v>
       </c>
       <c r="B26" s="10" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
       <c r="C26" s="10" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
     </row>
     <row r="27" spans="1:3" ht="30" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>132</v>
+        <v>128</v>
       </c>
       <c r="B27" s="10" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
       <c r="C27" s="10" t="s">
-        <v>231</v>
+        <v>227</v>
       </c>
     </row>
     <row r="28" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>133</v>
+        <v>129</v>
       </c>
       <c r="B28" s="10" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="C28" s="10" t="s">
-        <v>232</v>
+        <v>228</v>
       </c>
     </row>
     <row r="29" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>134</v>
+        <v>130</v>
       </c>
       <c r="B29" s="10" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="C29" s="10" t="s">
-        <v>233</v>
+        <v>229</v>
       </c>
     </row>
     <row r="30" spans="1:3" x14ac:dyDescent="0.25">
@@ -2372,7 +2587,7 @@
     </row>
     <row r="31" spans="1:3" s="14" customFormat="1" ht="90" x14ac:dyDescent="0.25">
       <c r="B31" s="29" t="s">
-        <v>216</v>
+        <v>212</v>
       </c>
       <c r="C31" s="15"/>
     </row>
@@ -2382,13 +2597,13 @@
     </row>
     <row r="33" spans="1:3" s="5" customFormat="1" ht="91.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B33" s="20" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="C33" s="6"/>
     </row>
     <row r="34" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>135</v>
+        <v>131</v>
       </c>
       <c r="B34" s="4" t="s">
         <v>16</v>
@@ -2397,7 +2612,7 @@
     </row>
     <row r="35" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
-        <v>136</v>
+        <v>132</v>
       </c>
       <c r="B35" s="4" t="s">
         <v>17</v>
@@ -2406,7 +2621,7 @@
     </row>
     <row r="36" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
-        <v>137</v>
+        <v>133</v>
       </c>
       <c r="B36" s="4" t="s">
         <v>43</v>
@@ -2415,29 +2630,29 @@
     </row>
     <row r="37" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
-        <v>138</v>
+        <v>134</v>
       </c>
       <c r="B37" s="10" t="s">
-        <v>111</v>
+        <v>107</v>
       </c>
       <c r="C37" s="10" t="s">
-        <v>223</v>
+        <v>219</v>
       </c>
     </row>
     <row r="38" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
-        <v>139</v>
+        <v>135</v>
       </c>
       <c r="B38" s="10" t="s">
-        <v>112</v>
+        <v>108</v>
       </c>
       <c r="C38" s="10" t="s">
-        <v>224</v>
+        <v>220</v>
       </c>
     </row>
     <row r="39" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
-        <v>140</v>
+        <v>136</v>
       </c>
       <c r="B39" s="4" t="s">
         <v>42</v>
@@ -2446,94 +2661,94 @@
     </row>
     <row r="40" spans="1:3" s="5" customFormat="1" ht="48.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B40" s="20" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="C40" s="6"/>
     </row>
     <row r="41" spans="1:3" ht="30" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
-        <v>141</v>
+        <v>137</v>
       </c>
       <c r="B41" s="10" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="C41" s="10"/>
     </row>
     <row r="42" spans="1:3" ht="45" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
-        <v>226</v>
+        <v>222</v>
       </c>
       <c r="B42" s="10" t="s">
-        <v>234</v>
+        <v>230</v>
       </c>
       <c r="C42" s="10" t="s">
-        <v>239</v>
+        <v>235</v>
       </c>
     </row>
     <row r="43" spans="1:3" ht="45" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
-        <v>142</v>
+        <v>138</v>
       </c>
       <c r="B43" s="10" t="s">
-        <v>113</v>
+        <v>109</v>
       </c>
       <c r="C43" s="10" t="s">
-        <v>235</v>
+        <v>231</v>
       </c>
     </row>
     <row r="44" spans="1:3" ht="47.25" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
-        <v>143</v>
+        <v>139</v>
       </c>
       <c r="B44" s="10" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="C44" s="10" t="s">
-        <v>241</v>
+        <v>237</v>
       </c>
     </row>
     <row r="45" spans="1:3" ht="30" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
-        <v>144</v>
+        <v>140</v>
       </c>
       <c r="B45" s="10" t="s">
         <v>36</v>
       </c>
       <c r="C45" s="10" t="s">
-        <v>227</v>
+        <v>223</v>
       </c>
     </row>
     <row r="46" spans="1:3" ht="30" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
-        <v>145</v>
+        <v>141</v>
       </c>
       <c r="B46" s="10" t="s">
-        <v>228</v>
+        <v>224</v>
       </c>
       <c r="C46" s="10" t="s">
-        <v>240</v>
+        <v>236</v>
       </c>
     </row>
     <row r="47" spans="1:3" s="5" customFormat="1" ht="54.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B47" s="20" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="C47" s="6"/>
     </row>
     <row r="48" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
-        <v>146</v>
+        <v>142</v>
       </c>
       <c r="B48" s="10" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="C48" s="38" t="s">
-        <v>229</v>
+        <v>225</v>
       </c>
     </row>
     <row r="49" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A49" t="s">
-        <v>147</v>
+        <v>143</v>
       </c>
       <c r="B49" s="4" t="s">
         <v>22</v>
@@ -2542,7 +2757,7 @@
     </row>
     <row r="50" spans="1:3" ht="30" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
-        <v>148</v>
+        <v>144</v>
       </c>
       <c r="B50" s="4" t="s">
         <v>28</v>
@@ -2551,210 +2766,210 @@
     </row>
     <row r="51" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
-        <v>149</v>
+        <v>145</v>
       </c>
       <c r="B51" s="4" t="s">
         <v>23</v>
       </c>
       <c r="C51" s="10" t="s">
-        <v>236</v>
+        <v>232</v>
       </c>
     </row>
     <row r="52" spans="1:3" ht="45" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
-        <v>150</v>
+        <v>146</v>
       </c>
       <c r="B52" s="4" t="s">
         <v>39</v>
       </c>
       <c r="C52" s="10" t="s">
-        <v>237</v>
+        <v>233</v>
       </c>
     </row>
     <row r="53" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
-        <v>151</v>
+        <v>147</v>
       </c>
       <c r="B53" s="4" t="s">
         <v>25</v>
       </c>
       <c r="C53" s="10" t="s">
-        <v>237</v>
+        <v>233</v>
       </c>
     </row>
     <row r="54" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
-        <v>152</v>
+        <v>148</v>
       </c>
       <c r="B54" s="4" t="s">
         <v>24</v>
       </c>
       <c r="C54" s="10" t="s">
-        <v>237</v>
+        <v>233</v>
       </c>
     </row>
     <row r="55" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
-        <v>153</v>
+        <v>149</v>
       </c>
       <c r="B55" s="3" t="s">
         <v>18</v>
       </c>
       <c r="C55" s="10" t="s">
-        <v>237</v>
+        <v>233</v>
       </c>
     </row>
     <row r="56" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
-        <v>154</v>
+        <v>150</v>
       </c>
       <c r="B56" s="3" t="s">
         <v>19</v>
       </c>
       <c r="C56" s="10" t="s">
-        <v>237</v>
+        <v>233</v>
       </c>
     </row>
     <row r="57" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
-        <v>155</v>
+        <v>151</v>
       </c>
       <c r="B57" s="4" t="s">
         <v>26</v>
       </c>
       <c r="C57" s="10" t="s">
-        <v>237</v>
+        <v>233</v>
       </c>
     </row>
     <row r="58" spans="1:3" ht="30" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
-        <v>156</v>
+        <v>152</v>
       </c>
       <c r="B58" s="4" t="s">
         <v>40</v>
       </c>
       <c r="C58" s="10" t="s">
-        <v>237</v>
+        <v>233</v>
       </c>
     </row>
     <row r="59" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
-        <v>157</v>
+        <v>153</v>
       </c>
       <c r="B59" s="4" t="s">
         <v>27</v>
       </c>
       <c r="C59" s="10" t="s">
-        <v>237</v>
+        <v>233</v>
       </c>
     </row>
     <row r="60" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
-        <v>158</v>
+        <v>154</v>
       </c>
       <c r="B60" s="10" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
       <c r="C60" s="10" t="s">
-        <v>237</v>
+        <v>233</v>
       </c>
     </row>
     <row r="61" spans="1:3" ht="33" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
-        <v>159</v>
+        <v>155</v>
       </c>
       <c r="B61" s="10" t="s">
-        <v>225</v>
+        <v>221</v>
       </c>
       <c r="C61" s="10" t="s">
-        <v>238</v>
+        <v>234</v>
       </c>
     </row>
     <row r="62" spans="1:3" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="C62" s="19" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
     </row>
     <row r="63" spans="1:3" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B63" s="19" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
     </row>
     <row r="64" spans="1:3" ht="409.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A64" s="22" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="B64" s="23" t="s">
         <v>7</v>
       </c>
       <c r="C64" s="23" t="s">
-        <v>110</v>
+        <v>106</v>
       </c>
     </row>
     <row r="65" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A65" s="24" t="s">
-        <v>160</v>
+        <v>156</v>
       </c>
       <c r="B65" s="25" t="s">
-        <v>209</v>
+        <v>205</v>
       </c>
       <c r="C65" s="25" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
     </row>
     <row r="66" spans="1:3" ht="30" x14ac:dyDescent="0.25">
       <c r="A66" s="24" t="s">
-        <v>161</v>
+        <v>157</v>
       </c>
       <c r="B66" s="25" t="s">
-        <v>210</v>
+        <v>206</v>
       </c>
       <c r="C66" s="25" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
     </row>
     <row r="67" spans="1:3" ht="30" x14ac:dyDescent="0.25">
       <c r="A67" s="24" t="s">
-        <v>162</v>
+        <v>158</v>
       </c>
       <c r="B67" s="25" t="s">
-        <v>211</v>
+        <v>207</v>
       </c>
       <c r="C67" s="25" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
     </row>
     <row r="68" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A68" s="24" t="s">
-        <v>163</v>
+        <v>159</v>
       </c>
       <c r="B68" s="25" t="s">
-        <v>212</v>
+        <v>208</v>
       </c>
       <c r="C68" s="25" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
     </row>
     <row r="69" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A69" s="24" t="s">
-        <v>165</v>
+        <v>161</v>
       </c>
       <c r="B69" s="25" t="s">
-        <v>213</v>
+        <v>209</v>
       </c>
       <c r="C69" s="25" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
     </row>
     <row r="70" spans="1:3" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A70" s="24" t="s">
-        <v>164</v>
+        <v>160</v>
       </c>
       <c r="B70" s="25" t="s">
-        <v>214</v>
+        <v>210</v>
       </c>
       <c r="C70" s="25" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
     </row>
     <row r="71" spans="1:3" s="5" customFormat="1" x14ac:dyDescent="0.25">
@@ -2769,7 +2984,7 @@
     </row>
     <row r="73" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A73" t="s">
-        <v>168</v>
+        <v>164</v>
       </c>
       <c r="B73" s="3" t="s">
         <v>20</v>
@@ -2777,7 +2992,7 @@
     </row>
     <row r="74" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A74" t="s">
-        <v>167</v>
+        <v>163</v>
       </c>
       <c r="B74" s="3" t="s">
         <v>41</v>
@@ -2785,7 +3000,7 @@
     </row>
     <row r="75" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A75" t="s">
-        <v>166</v>
+        <v>162</v>
       </c>
       <c r="B75" s="3" t="s">
         <v>21</v>
@@ -2793,20 +3008,20 @@
     </row>
     <row r="78" spans="1:3" s="5" customFormat="1" ht="120" x14ac:dyDescent="0.25">
       <c r="B78" s="12" t="s">
-        <v>109</v>
+        <v>242</v>
       </c>
       <c r="C78" s="13" t="s">
-        <v>46</v>
+        <v>243</v>
       </c>
     </row>
     <row r="79" spans="1:3" x14ac:dyDescent="0.25">
       <c r="C79" s="39" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
     </row>
     <row r="80" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A80" t="s">
-        <v>169</v>
+        <v>165</v>
       </c>
       <c r="B80" s="9" t="s">
         <v>34</v>
@@ -2815,7 +3030,7 @@
     </row>
     <row r="81" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A81" t="s">
-        <v>170</v>
+        <v>166</v>
       </c>
       <c r="B81" s="9" t="s">
         <v>29</v>
@@ -2824,7 +3039,7 @@
     </row>
     <row r="82" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A82" t="s">
-        <v>171</v>
+        <v>167</v>
       </c>
       <c r="B82" s="9" t="s">
         <v>30</v>
@@ -2833,7 +3048,7 @@
     </row>
     <row r="83" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A83" t="s">
-        <v>172</v>
+        <v>168</v>
       </c>
       <c r="B83" s="9" t="s">
         <v>31</v>
@@ -2842,7 +3057,7 @@
     </row>
     <row r="84" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A84" t="s">
-        <v>173</v>
+        <v>169</v>
       </c>
       <c r="B84" s="8" t="s">
         <v>35</v>
@@ -2851,7 +3066,7 @@
     </row>
     <row r="85" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A85" t="s">
-        <v>174</v>
+        <v>170</v>
       </c>
       <c r="B85" s="8" t="s">
         <v>32</v>
@@ -2860,7 +3075,7 @@
     </row>
     <row r="86" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A86" t="s">
-        <v>175</v>
+        <v>171</v>
       </c>
       <c r="B86" s="7" t="s">
         <v>33</v>
@@ -2869,308 +3084,308 @@
     </row>
     <row r="87" spans="1:3" ht="30" x14ac:dyDescent="0.25">
       <c r="A87" t="s">
-        <v>176</v>
+        <v>172</v>
       </c>
       <c r="B87" s="4" t="s">
         <v>38</v>
       </c>
       <c r="C87" s="40"/>
     </row>
-    <row r="90" spans="1:3" s="5" customFormat="1" ht="75" x14ac:dyDescent="0.25">
+    <row r="90" spans="1:3" s="5" customFormat="1" ht="105" x14ac:dyDescent="0.25">
       <c r="B90" s="20" t="s">
-        <v>108</v>
+        <v>241</v>
       </c>
       <c r="C90" s="21" t="s">
-        <v>48</v>
+        <v>244</v>
       </c>
     </row>
     <row r="92" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A92" t="s">
-        <v>177</v>
+        <v>173</v>
       </c>
       <c r="B92" s="10" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="C92" s="41" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
     </row>
     <row r="93" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A93" t="s">
-        <v>178</v>
+        <v>174</v>
       </c>
       <c r="B93" s="10" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="C93" s="41"/>
     </row>
     <row r="94" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A94" t="s">
-        <v>179</v>
+        <v>175</v>
       </c>
       <c r="B94" s="10" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="C94" s="41"/>
     </row>
     <row r="95" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A95" t="s">
-        <v>188</v>
+        <v>184</v>
       </c>
       <c r="B95" s="10" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="C95" s="41"/>
     </row>
     <row r="96" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A96" t="s">
-        <v>189</v>
+        <v>185</v>
       </c>
       <c r="B96" s="10" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="C96" s="41"/>
     </row>
     <row r="97" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A97" t="s">
-        <v>190</v>
+        <v>186</v>
       </c>
       <c r="B97" s="10" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="C97" s="41"/>
     </row>
     <row r="98" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A98" t="s">
-        <v>191</v>
+        <v>187</v>
       </c>
       <c r="B98" s="10" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="C98" s="41"/>
     </row>
     <row r="99" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A99" t="s">
-        <v>192</v>
+        <v>188</v>
       </c>
       <c r="B99" s="10" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="C99" s="41"/>
     </row>
     <row r="100" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A100" t="s">
-        <v>193</v>
+        <v>189</v>
       </c>
       <c r="B100" s="3" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="C100" s="41"/>
     </row>
     <row r="101" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A101" t="s">
-        <v>194</v>
+        <v>190</v>
       </c>
       <c r="B101" s="3" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="C101" s="41"/>
     </row>
     <row r="102" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A102" t="s">
-        <v>195</v>
+        <v>191</v>
       </c>
       <c r="B102" s="3" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="C102" s="41"/>
     </row>
     <row r="103" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A103" t="s">
-        <v>196</v>
+        <v>192</v>
       </c>
       <c r="B103" s="3" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="C103" s="41"/>
     </row>
     <row r="104" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A104" t="s">
-        <v>197</v>
+        <v>193</v>
       </c>
       <c r="B104" s="3" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="C104" s="41"/>
     </row>
     <row r="105" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A105" t="s">
-        <v>198</v>
+        <v>194</v>
       </c>
       <c r="B105" s="3" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="C105" s="41"/>
     </row>
     <row r="106" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A106" t="s">
-        <v>199</v>
+        <v>195</v>
       </c>
       <c r="B106" s="3" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="C106" s="41"/>
     </row>
     <row r="107" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A107" t="s">
-        <v>200</v>
+        <v>196</v>
       </c>
       <c r="B107" s="3" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="C107" s="41"/>
     </row>
     <row r="108" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A108" t="s">
-        <v>201</v>
+        <v>197</v>
       </c>
       <c r="B108" s="10" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="C108" s="41"/>
     </row>
     <row r="109" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A109" t="s">
-        <v>202</v>
+        <v>198</v>
       </c>
       <c r="B109" s="10" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="C109" s="41"/>
     </row>
     <row r="110" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A110" t="s">
-        <v>203</v>
+        <v>199</v>
       </c>
       <c r="B110" s="10" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="C110" s="41"/>
     </row>
     <row r="111" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A111" t="s">
-        <v>204</v>
+        <v>200</v>
       </c>
       <c r="B111" s="10" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="C111" s="41"/>
     </row>
     <row r="112" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A112" t="s">
-        <v>205</v>
+        <v>201</v>
       </c>
       <c r="B112" s="10" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="C112" s="41"/>
     </row>
     <row r="113" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A113" t="s">
-        <v>206</v>
+        <v>202</v>
       </c>
       <c r="B113" s="10" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="C113" s="41"/>
     </row>
     <row r="114" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A114" t="s">
-        <v>207</v>
+        <v>203</v>
       </c>
       <c r="B114" s="10" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="C114" s="41"/>
     </row>
     <row r="115" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A115" t="s">
-        <v>208</v>
+        <v>204</v>
       </c>
       <c r="B115" s="10" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="C115" s="41"/>
     </row>
     <row r="116" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A116" t="s">
-        <v>187</v>
+        <v>183</v>
       </c>
       <c r="B116" s="3" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="C116" s="41"/>
     </row>
     <row r="117" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A117" t="s">
-        <v>186</v>
+        <v>182</v>
       </c>
       <c r="B117" s="3" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="C117" s="41"/>
     </row>
     <row r="118" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A118" t="s">
-        <v>185</v>
+        <v>181</v>
       </c>
       <c r="B118" s="3" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="C118" s="41"/>
     </row>
     <row r="119" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A119" t="s">
-        <v>184</v>
+        <v>180</v>
       </c>
       <c r="B119" s="3" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="C119" s="41"/>
     </row>
     <row r="120" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A120" t="s">
-        <v>183</v>
+        <v>179</v>
       </c>
       <c r="B120" s="3" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="C120" s="41"/>
     </row>
     <row r="121" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A121" t="s">
-        <v>182</v>
+        <v>178</v>
       </c>
       <c r="B121" s="3" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="C121" s="41"/>
     </row>
     <row r="122" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A122" t="s">
-        <v>181</v>
+        <v>177</v>
       </c>
       <c r="B122" s="3" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="C122" s="41"/>
     </row>
     <row r="123" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A123" t="s">
-        <v>180</v>
+        <v>176</v>
       </c>
       <c r="B123" s="3" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="C123" s="41"/>
     </row>

</xml_diff>